<commit_message>
TBCP: add Master and DEPC agreements (02.01, 02.02)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NhaKeVxjNyTBn6poC6zJrZ
</commit_message>
<xml_diff>
--- a/Lumbee_RIVR_TBCP_Agreement_Package/01_Phase1_Diligence/01_Source_and_Assumptions_Register.xlsx
+++ b/Lumbee_RIVR_TBCP_Agreement_Package/01_Phase1_Diligence/01_Source_and_Assumptions_Register.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,14 +69,6 @@
     <font>
       <b val="1"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -162,7 +154,7 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">

</xml_diff>

<commit_message>
TBCP: add operational forms (04), README, consistency pass (11/0/0), party-line injection
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NhaKeVxjNyTBn6poC6zJrZ
</commit_message>
<xml_diff>
--- a/Lumbee_RIVR_TBCP_Agreement_Package/01_Phase1_Diligence/01_Source_and_Assumptions_Register.xlsx
+++ b/Lumbee_RIVR_TBCP_Agreement_Package/01_Phase1_Diligence/01_Source_and_Assumptions_Register.xlsx
@@ -550,6 +550,14 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Parties: Lumbee Tribe of North Carolina (the “Lumbee Tribe”); LREMC Technologies, LLC d/b/a RIVR Tech (“RIVR Tech”); Lumbee River Electric Membership Corporation d/b/a Lumbee River EMC (“LREMC”), separate asset owner.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -626,6 +634,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>

</xml_diff>